<commit_message>
fix: update password auto create for student
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/templates/download/student_import_template.xlsx
+++ b/backend/src/main/resources/templates/download/student_import_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\lab_supervise\backend\src\main\resources\templates\download\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33BD75BE-D2A4-47E7-A94E-471268105569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{927027D1-30B5-4DB0-A47E-20506A97C6C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>STT</t>
   </si>
@@ -34,18 +34,6 @@
   </si>
   <si>
     <t>Họ Tên</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Số điện thoại</t>
-  </si>
-  <si>
-    <t>Ngày sinh</t>
-  </si>
-  <si>
-    <t>Quê quán</t>
   </si>
   <si>
     <t>Lớp quản lý</t>
@@ -405,20 +393,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="27.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="18.33203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="31.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="23.77734375" style="2" customWidth="1"/>
-    <col min="7" max="8" width="21.88671875" style="2" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="27.28515625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="31.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="23.7109375" style="2" customWidth="1"/>
+    <col min="7" max="8" width="21.85546875" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="36.6" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -429,30 +417,14 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>